<commit_message>
Introduction vérif elastique IFB-A Introduction lSlimMixte
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS SFS02/Cas SFS02.xlsx
+++ b/VALIDATION/CAS SFS02/Cas SFS02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS SFS02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF30192-FD13-4E86-B342-38AC6A211A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8517F67-C611-468C-958A-29FCCE0E8698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -59,6 +59,7 @@
     <definedName name="hb">Feuil1!$D$12</definedName>
     <definedName name="Ht">Feuil1!$D$15</definedName>
     <definedName name="hw">Feuil1!$D$8</definedName>
+    <definedName name="hwe">Feuil1!$N$45</definedName>
     <definedName name="hwP">Feuil1!$D$16</definedName>
     <definedName name="IncertieCM">Feuil1!$N$29</definedName>
     <definedName name="InertieY_MM4">Feuil1!$N$28</definedName>
@@ -134,7 +135,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="156">
   <si>
     <t>hw</t>
   </si>
@@ -599,6 +600,9 @@
   </si>
   <si>
     <t>w-inf</t>
+  </si>
+  <si>
+    <t>Hauteur de l'élément âme</t>
   </si>
 </sst>
 </file>
@@ -611,7 +615,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -631,6 +635,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -903,7 +914,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1152,6 +1163,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2381,7 +2398,7 @@
       </c>
       <c r="J36" s="52">
         <f>MEd_U1/MplRd</f>
-        <v>0.68444711032113492</v>
+        <v>0.74028353165455463</v>
       </c>
       <c r="M36" s="41" t="s">
         <v>92</v>
@@ -2606,13 +2623,23 @@
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
-      <c r="M45" t="s">
-        <v>152</v>
+      <c r="M45" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="N45" s="6">
+        <f>hwP</f>
+        <v>206</v>
+      </c>
+      <c r="O45" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C46" s="3"/>
       <c r="D46" s="4"/>
+      <c r="M46" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="47" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C47" s="3" t="s">
@@ -2628,6 +2655,10 @@
         <v>48</v>
       </c>
       <c r="N47" s="52">
+        <f>(P35+P36+P37-P40)/2/P37</f>
+        <v>5.2838812974922822E-2</v>
+      </c>
+      <c r="Q47" s="52">
         <f>(P35+P36+P37-P40)/2/P37</f>
         <v>5.2838812974922822E-2</v>
       </c>
@@ -2639,11 +2670,15 @@
         <v>49</v>
       </c>
       <c r="N48" s="53">
-        <f>pANP*(hw-rr)</f>
-        <v>17.172614216849919</v>
+        <f>pANP*(hwe)</f>
+        <v>10.884795472834101</v>
       </c>
       <c r="O48" t="s">
         <v>2</v>
+      </c>
+      <c r="S48">
+        <f>(1-pANP)*(hwP-rr)/2</f>
+        <v>84.770926238744408</v>
       </c>
     </row>
     <row r="49" spans="3:21" x14ac:dyDescent="0.25">
@@ -2674,6 +2709,10 @@
       </c>
       <c r="E50" t="s">
         <v>63</v>
+      </c>
+      <c r="S50">
+        <f>hwP-rr</f>
+        <v>179</v>
       </c>
     </row>
     <row r="51" spans="3:21" x14ac:dyDescent="0.25">
@@ -2733,11 +2772,14 @@
       </c>
       <c r="P52" s="67">
         <f>O52-zANP</f>
-        <v>200.82738578315008</v>
+        <v>207.1152045271659</v>
       </c>
       <c r="Q52" s="87">
         <f>N52*ABS(P52/1000)</f>
-        <v>498.85522628534477</v>
+        <v>514.47416804548004</v>
+      </c>
+      <c r="R52" s="102">
+        <v>514.47</v>
       </c>
       <c r="T52" s="101">
         <f>(1-T53)-T53</f>
@@ -2779,11 +2821,14 @@
       </c>
       <c r="P53" s="68">
         <f>O53-zANP</f>
-        <v>182.79645143161477</v>
+        <v>189.08427017563059</v>
       </c>
       <c r="Q53" s="89">
         <f t="shared" ref="Q53:Q56" si="9">N53*ABS(P53/1000)</f>
-        <v>19.732304747973814</v>
+        <v>20.411055099445264</v>
+      </c>
+      <c r="R53" s="102">
+        <v>20.41</v>
       </c>
       <c r="T53" s="101">
         <f>1-T54</f>
@@ -2808,17 +2853,18 @@
         <v>908.74906508527522</v>
       </c>
       <c r="O54" s="88">
-        <f>(hw-rr)-(1-pANP)*(hw-rr)/2</f>
-        <v>171.08630710842496</v>
+        <f>(hwe)-(1-pANP)*(hwe)/2</f>
+        <v>108.44239773641705</v>
       </c>
       <c r="P54" s="68">
         <f>O54-zANP</f>
-        <v>153.91369289157504</v>
-      </c>
-      <c r="Q54" s="89">
+        <v>97.55760226358295</v>
+      </c>
+      <c r="Q54" s="103">
         <f t="shared" si="9"/>
-        <v>139.86892451904097</v>
-      </c>
+        <v>88.655379848992141</v>
+      </c>
+      <c r="R54" s="102"/>
       <c r="S54" s="6">
         <v>105</v>
       </c>
@@ -2857,16 +2903,19 @@
         <v>50.69593491472483</v>
       </c>
       <c r="O55" s="88">
-        <f>(pANP)*(hw-rr)/2</f>
-        <v>8.5863071084249594</v>
+        <f>(pANP)*(hwe)/2</f>
+        <v>5.4423977364170506</v>
       </c>
       <c r="P55" s="68">
         <f>O55-zANP</f>
-        <v>-8.5863071084249594</v>
-      </c>
-      <c r="Q55" s="89">
+        <v>-5.4423977364170506</v>
+      </c>
+      <c r="Q55" s="103">
         <f t="shared" si="9"/>
-        <v>0.4352908663265509</v>
+        <v>0.27590744142544454</v>
+      </c>
+      <c r="R55" s="102">
+        <v>88.93</v>
       </c>
       <c r="U55" s="75">
         <f>T54*P37</f>
@@ -2890,11 +2939,14 @@
       </c>
       <c r="P56" s="73">
         <f>O56-zANP</f>
-        <v>-27.172614216849919</v>
+        <v>-20.884795472834099</v>
       </c>
       <c r="Q56" s="91">
         <f t="shared" si="9"/>
-        <v>93.745519048132209</v>
+        <v>72.052544381277642</v>
+      </c>
+      <c r="R56" s="102">
+        <v>72.040000000000006</v>
       </c>
       <c r="U56" s="75"/>
     </row>
@@ -2904,7 +2956,7 @@
       <c r="J57" s="4"/>
       <c r="Q57" s="85">
         <f>SUM(Q52:Q56)</f>
-        <v>752.63726546681835</v>
+        <v>695.86905481662052</v>
       </c>
       <c r="U57" s="75">
         <f>U54-U55</f>
@@ -2924,7 +2976,7 @@
       </c>
       <c r="Q59" s="76">
         <f>Q57</f>
-        <v>752.63726546681835</v>
+        <v>695.86905481662052</v>
       </c>
       <c r="R59" t="s">
         <v>18</v>

</xml_diff>